<commit_message>
feat: enhance invoice filters with year selection and dynamic search placeholders
</commit_message>
<xml_diff>
--- a/public/templates/apartments_template.xlsx
+++ b/public/templates/apartments_template.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="00"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -64,8 +65,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,6 +400,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,7 +422,7 @@
         <v>Area (Sqft)</v>
       </c>
       <c r="E1" t="str">
-        <v>Type</v>
+        <v>Type (BHK)</v>
       </c>
     </row>
     <row r="2">
@@ -423,14 +432,14 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" t="str">
-        <v>01</v>
+      <c r="C2" s="1">
+        <v>1</v>
       </c>
       <c r="D2">
         <v>1200</v>
       </c>
-      <c r="E2" t="str">
-        <v>2BHK</v>
+      <c r="E2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance import modal with async file upload handling and loading state
</commit_message>
<xml_diff>
--- a/public/templates/apartments_template.xlsx
+++ b/public/templates/apartments_template.xlsx
@@ -401,11 +401,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>